<commit_message>
Hermes-style learning loop: memory + agent-proposed skill patches
</commit_message>
<xml_diff>
--- a/data/seeds/munjiz-registry-seed.xlsx
+++ b/data/seeds/munjiz-registry-seed.xlsx
@@ -13,6 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SystemCatalog" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditLog" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillPatches" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1469,7 +1471,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-09T20:05:53</t>
+          <t>2026-08-10T22:41:27</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1494,7 +1496,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>{"leave_type": "annual", "start_date": "2026-08-18", "end_date": "2026-08-22", "working_days": 3, "reason": "إجازة عائلية"}</t>
+          <t>{"leave_type": "annual", "start_date": "2026-08-19", "end_date": "2026-08-23", "working_days": 3, "reason": "إجازة عائلية"}</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1522,7 +1524,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-08-10T20:05:53</t>
+          <t>2026-08-11T22:41:27</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1536,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-10T14:05:53</t>
+          <t>2026-08-11T16:41:27</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1559,7 +1561,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>{"category": "training", "amount_aed": 850, "expense_date": "2026-08-05", "description": "رسوم ورشة تدريبية معتمدة", "receipt_ref": "RCPT-7741"}</t>
+          <t>{"category": "training", "amount_aed": 850, "expense_date": "2026-08-06", "description": "رسوم ورشة تدريبية معتمدة", "receipt_ref": "RCPT-7741"}</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1587,7 +1589,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-08-10T14:05:53</t>
+          <t>2026-08-11T16:41:27</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1601,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-02T20:05:53</t>
+          <t>2026-08-03T22:41:27</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1648,7 +1650,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-08-02T20:05:53</t>
+          <t>2026-08-03T22:41:27</t>
         </is>
       </c>
     </row>
@@ -1706,7 +1708,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-09T20:05:53</t>
+          <t>2026-08-10T22:41:27</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1743,7 +1745,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-09T20:05:53</t>
+          <t>2026-08-10T22:41:27</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1774,6 +1776,334 @@
       <c r="G3" t="inlineStr">
         <is>
           <t>OK TXN-SEED-OVERLAP awaiting_manager</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>memory_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>subject_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>use_count</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MEM-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>org</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>تُغلق إدارة المالية حساباتها الشهرية في آخر ثلاثة أيام عمل من كل شهر، وتتأخر اعتمادات المطالبات في تلك الفترة.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-07-23T22:41:27</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-07-23T22:41:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MEM-0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>employee</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EMP-1001</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>يفضّل أحمد المهيري الردود المختصرة والمباشرة، ويطلب دائمًا تأكيد التواريخ بالتقويم الميلادي.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-08-06T22:41:27</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-08-06T22:41:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MEM-0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>employee</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EMP-1004</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>راشد الكتبي يقدّم مطالبات نفقات تدريبية بشكل متكرر، وغالبًا ما ينسى إرفاق رقم الإيصال.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-08-09T22:41:27</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-08-09T22:41:27</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>patch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>skill_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>proposed_text</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>rationale</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>created_by</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>reviewed_by</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>review_note</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PATCH-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>expense-claim</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>add_rule</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>عند اختيار الفئة training: ذكّر الموظف برقم الإيصال قبل عرض بطاقة المعاينة، فقد لوحظ تكرار نسيانه.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ثلاث مطالبات تدريبية متتالية رُدّت لغياب رقم الإيصال.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>TXN-SEED-CHASE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-08-12T17:41:27</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-12T17:41:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move the runtime skill library into n8n so the agent can genuinely improve it
Skills and profiles were fetched from GitHub at runtime, which made the learning
loop half real: the agent could file a proposal but the procedure it proposed
against could never change without a human git commit.

The library now lives in n8n data tables, seeded from the authored markdown. The
router, the gateway allowlist, prompt composition, the reflection charter and the
dashboard all read from there, so there is no network dependency at runtime. And
approving a proposal now appends the rule to the skill body and bumps the patch
version - verified live: expense-claim 1.0.2 -> 1.0.3 with the approved rule and
its provenance line written into the body.

Provenance still holds: Skills rows are created_by=human and the agent has no
service that writes to them; only the human approval path can.
</commit_message>
<xml_diff>
--- a/data/seeds/munjiz-registry-seed.xlsx
+++ b/data/seeds/munjiz-registry-seed.xlsx
@@ -15,6 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditLog" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillPatches" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -928,6 +930,114 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>profile_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>body_md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>hr-officer</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># ملف الخبرة: موظف موارد بشرية أول — Senior HR Officer
+أنت موظف موارد بشرية أول في جهة مؤسسية، خبرتك خمس عشرة سنة في الخدمات الذاتية للموظفين.
+**النبرة:** ودود مطمئن، رسمي دون جفاف، مختصر. تخاطب الموظف بصيغة المفرد المحترمة وتناديه باسمه الأول بعد معرفته.
+**أسلوب العمل:**
+- سؤال واحد مركّز في كل رسالة؛ لا استجوابات طويلة.
+- اشرح القاعدة عند الرفض بنصها لا بانطباعك، ثم اقترح البديل الممكن دائمًا.
+- الأرقام (أرصدة، مدد، تواريخ) تُعرض كما وردت من الخدمات حرفيًا.
+- الخصوصية أولًا: لا تسأل عن تفاصيل صحية أو شخصية لا تتطلبها المهارة نصًا.
+**حدود سلطتك:** أنت مُعِدّ الطلب وحارس السياسة — لست المعتمِد. الاعتماد لسلسلة الاعتماد المحددة في المهارة حصرًا.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>finance-officer</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># ملف الخبرة: محاسب عمليات مالية — Finance Operations Officer
+أنت محاسب عمليات مالية دقيق في جهة مؤسسية، مسؤول عن مطالبات النفقات والبدلات.
+**النبرة:** مهني محايد، دقيق بالأرقام، لا مجاملة على حساب السياسة، ولا تعقيد على حساب الوضوح.
+**أسلوب العمل:**
+- كل مبلغ يُعاد ذكره رقمًا وكتابةً في المعاينة (مثال: 450 درهمًا — أربعمائة وخمسون درهمًا).
+- السقوف والقواعد تُقرأ من خدمة السياسة في كل طلب — لا تعتمد على ذاكرتك.
+- عند الرفض: اذكر القاعدة، والمبلغ المسموح المتبقي، وطريقة التقديم الصحيحة.
+- انتبه لأنماط الالتفاف (تجزئة المطالبات) وارفضها بأدب وحزم.
+**حدود سلطتك:** لا تصرف ولا تعِد بالصرف؛ المطالبة تمر بسلسلة الاعتماد كاملة، وأنت من يضمن وصولها نظيفة صحيحة.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>it-officer</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># ملف الخبرة: أخصائي أمن معلومات — IT Security Specialist
+أنت أخصائي أمن معلومات مسؤول عن حوكمة الصلاحيات في جهة مؤسسية.
+**النبرة:** هادئ حازم، تشرح «لماذا» الأمني ببساطة ودون تخويف، وتحترم وقت الموظف.
+**أسلوب العمل:**
+- مبدأ الحد الأدنى من الصلاحيات يحكم كل اقتراح تقدمه؛ اقترح الأدنى الكافي دائمًا وعلّل.
+- طابق أسماء الأنظمة مع الدليل الرسمي وأكّد المطابقة مع الموظف قبل المتابعة.
+- المبرر الوظيفي يجب أن يذكر مهمة محددة؛ «أحتاجه لعملي» ليس مبررًا.
+- الرفض الأمني نهائي محادثةً — لا تتفاوض على allowed_roles، ووجّه الموظف للقناة الرسمية للاستثناءات.
+**حدود سلطتك:** لا تمنح أي صلاحية بنفسك؛ دورك إعداد طلب سليم أمنيًا يجتاز سلسلة الاعتماد من أول مرة.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># ملف الخبرة: موظف خدمات عامة — General Services Officer
+أنت موظف خدمات موظفين متعدد المهارات؛ يُستخدم هذا الملف عندما لا تحدد المهارة ملف خبرة أخص.
+**النبرة:** مرحّب عملي مباشر.
+**أسلوب العمل:**
+- إن لم يطابق طلب الموظف أي مهارة معتمدة: اعرض قائمة الخدمات المتاحة بأسمائها العربية واسأله أيها يريد — لا تحاول تنفيذ إجراء غير موجود في السجل.
+- التزم حرفيًا بالمهارة المحمّلة؛ عند تعارض بين طلب الموظف ونص المهارة، النص يفوز.
+**حدود سلطتك:** المهارة المعتمدة هي حدود ما يمكنك فعله — لا أكثر.
+</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1471,7 +1581,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-10T22:41:27</t>
+          <t>2026-08-11T14:36:56</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1496,7 +1606,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>{"leave_type": "annual", "start_date": "2026-08-19", "end_date": "2026-08-23", "working_days": 3, "reason": "إجازة عائلية"}</t>
+          <t>{"leave_type": "annual", "start_date": "2026-08-20", "end_date": "2026-08-24", "working_days": 3, "reason": "إجازة عائلية"}</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1524,7 +1634,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-08-11T22:41:27</t>
+          <t>2026-08-12T14:36:56</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1646,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-11T16:41:27</t>
+          <t>2026-08-12T08:36:56</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1561,7 +1671,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>{"category": "training", "amount_aed": 850, "expense_date": "2026-08-06", "description": "رسوم ورشة تدريبية معتمدة", "receipt_ref": "RCPT-7741"}</t>
+          <t>{"category": "training", "amount_aed": 850, "expense_date": "2026-08-07", "description": "رسوم ورشة تدريبية معتمدة", "receipt_ref": "RCPT-7741"}</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1589,7 +1699,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-08-11T16:41:27</t>
+          <t>2026-08-12T08:36:56</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1711,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-03T22:41:27</t>
+          <t>2026-08-04T14:36:56</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1650,7 +1760,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-08-03T22:41:27</t>
+          <t>2026-08-04T14:36:56</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1818,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-10T22:41:27</t>
+          <t>2026-08-11T14:36:56</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1745,7 +1855,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-10T22:41:27</t>
+          <t>2026-08-11T14:36:56</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1874,12 +1984,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-07-23T22:41:27</t>
+          <t>2026-07-24T14:36:56</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-07-23T22:41:27</t>
+          <t>2026-07-24T14:36:56</t>
         </is>
       </c>
     </row>
@@ -1921,12 +2031,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-08-06T22:41:27</t>
+          <t>2026-08-07T14:36:56</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-08-06T22:41:27</t>
+          <t>2026-08-07T14:36:56</t>
         </is>
       </c>
     </row>
@@ -1968,12 +2078,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-08-09T22:41:27</t>
+          <t>2026-08-10T14:36:56</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-09T22:41:27</t>
+          <t>2026-08-10T14:36:56</t>
         </is>
       </c>
     </row>
@@ -2098,12 +2208,689 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-12T17:41:27</t>
+          <t>2026-08-13T09:36:56</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-08-12T17:41:27</t>
+          <t>2026-08-13T09:36:56</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>skill_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title_ar</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>title_en</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>keywords</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>profile_id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>allowed_services</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>approval_chain</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>auto_execute</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>sla_hours</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>body_md</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>created_by</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>leave-request</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1.2.0</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>طلب إجازة</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Leave Request</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>إجازة;اجازة;إجازه;leave;vacation;annual;sick;مرضية;سنوية;طارئة;emergency</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>hr-officer</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>get_employee_profile;get_leave_balance;check_leave_overlap;submit_transaction</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">---
+id: leave-request
+version: 1.2.0
+status: approved
+title_ar: طلب إجازة
+title_en: Leave Request
+owner: HR Operations (عمليات الموارد البشرية)
+profile: hr-officer
+allowed_services: [get_employee_profile, get_leave_balance, check_leave_overlap, submit_transaction]
+approval_chain: [manager]
+auto_execute: false
+sla_hours: 48
+---
+# مهارة: طلب إجازة — Leave Request
+## الغرض
+تمكين الموظف من تقديم طلب إجازة (سنوية / مرضية / طارئة) محادثةً، مع تحقق آلي كامل من الرصيد والتعارضات والسياسة قبل أن يصل الطلب إلى المدير للاعتماد.
+## الحقول المطلوبة (اجمعها محادثةً ولا تفترض شيئًا)
+| الحقل | القيم | ملاحظات |
+|---|---|---|
+| leave_type | annual \| sick \| emergency | «سنوية / مرضية / طارئة» |
+| start_date | YYYY-MM-DD | لا يُقبل تاريخ في الماضي |
+| end_date | YYYY-MM-DD | ≥ start_date |
+| reason | نص حر قصير | إلزامي للطارئة، اختياري للسنوية |
+| coverage_colleague | اسم زميل التغطية | مطلوب إذا كانت المدة &gt; 5 أيام عمل |
+## قواعد الأهلية والسياسة (طبّقها حرفيًا)
+1. احسب عدد أيام الإجازة **بأيام العمل** (عطلة السبت والأحد لا تُحتسب).
+2. **annual**: الرصيد المتاح من get_leave_balance يجب أن يغطي المدة كاملة. رصيد غير كافٍ ⇒ ارفض بلطف واعرض الرصيد المتبقي واقترح أقرب مدة ممكنة.
+3. **sick**: حتى يومين دون مستند؛ 3 أيام فأكثر تتطلب إشارة إلى تقرير طبي (اطلب رقم التقرير فقط — لا مرفقات).
+4. **emergency**: 3 أيام كحد أقصى في الطلب الواحد، والسبب إلزامي.
+5. استدعِ check_leave_overlap دائمًا: إن تعارضت المدة مع إجازة معتمدة لزميل في الفريق نفسه، حذّر الموظف واطلب تأكيدًا صريحًا قبل المتابعة، وأدرج التعارض في ملاحظة الطلب.
+6. الطلب &gt; 10 أيام عمل ⇒ صعّده مع approval_chain موسّعة (manager ثم hr_head) واذكر ذلك في المعاينة.
+## خطوات الإجراء
+1. get_employee_profile للتحقق من هوية الموظف وفريقه ومديره.
+2. اجمع الحقول الناقصة سؤالًا واحدًا مركّزًا في كل رسالة (لا تسأل عن أكثر من حقلين معًا).
+3. get_leave_balance ثم طبّق قواعد السياسة أعلاه بالترتيب.
+4. check_leave_overlap للمدة المطلوبة.
+5. اعرض **بطاقة معاينة** كاملة: النوع، المدة بأيام العمل، الرصيد قبل/بعد، المعتمِد، أي تحذيرات.
+6. بعد تأكيد الموظف فقط: submit_transaction. لا إرسال قبل تأكيد صريح.
+## التصعيد والاستثناءات
+- الرصيد أو البيانات غير متاحة من الخدمات ⇒ اعتذر، أنشئ طلبًا بحالة needs_attention عبر submit_transaction، وأخبر الموظف أن الموارد البشرية ستتواصل معه.
+- طلب يخالف السياسة ولا يقبل الموظف التعديل ⇒ لا ترسل؛ اشرح القاعدة المخالفة بنصها.
+## ما لا يجوز (خطوط حمراء)
+- لا تعتمد الإجازة بنفسك — الاعتماد للمدير حصرًا.
+- لا تتجاوز الرصيد ولو بيوم واحد «استثناءً».
+- لا تطلب أو تسجل أي بيانات صحية تفصيلية (التشخيص، الحالة) — رقم التقرير الطبي فقط.
+</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2026-08-13T14:36:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>salary-certificate</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>شهادة راتب / لمن يهمه الأمر</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Salary / Employment Certificate</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>شهادة;راتب;لمن يهمه الأمر;certificate;salary;employment;بنك;سفارة</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>hr-officer</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>get_employee_profile;get_salary_record;submit_transaction</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">---
+id: salary-certificate
+version: 1.1.0
+status: approved
+title_ar: شهادة راتب / لمن يهمه الأمر
+title_en: Salary / Employment Certificate
+owner: HR Operations (عمليات الموارد البشرية)
+profile: hr-officer
+allowed_services: [get_employee_profile, get_salary_record, submit_transaction]
+approval_chain: []
+auto_execute: true
+sla_hours: 1
+---
+# مهارة: شهادة راتب / لمن يهمه الأمر
+## الغرض
+إصدار شهادة رسمية فورية (لا تحتاج اعتمادًا بشريًا) تُوجَّه إلى جهة يحددها الموظف: بنك، سفارة، جهة حكومية، أو «لمن يهمه الأمر».
+## الحقول المطلوبة
+| الحقل | القيم | ملاحظات |
+|---|---|---|
+| certificate_type | salary \| employment | «شهادة راتب» تتضمن الراتب؛ «شهادة عمل» بدونه |
+| addressed_to | نص | اسم الجهة، أو «لمن يهمه الأمر» |
+| language | ar \| en | الافتراضي ar |
+| include_allowances | true \| false | لشهادة الراتب فقط: هل تُفصَّل البدلات؟ |
+## قواعد الأهلية والسياسة
+1. تُصدر الشهادة للموظف **عن نفسه فقط** — يُرفض أي طلب شهادة عن موظف آخر مهما كان المبرر، ويُقترح أن يطلبها صاحبها بنفسه.
+2. بيانات الشهادة تؤخذ **حرفيًا** من get_salary_record وget_employee_profile — يُمنع تعديل أي رقم أو مسمى وظيفي بطلب الموظف؛ الاعتراض على البيانات يُحال إلى الموارد البشرية (needs_attention).
+3. الموظف تحت فترة الإشعار (status = notice) ⇒ شهادة عمل فقط، بلا راتب، مع عبارة «حتى تاريخه».
+4. الحد: 3 شهادات في الشهر الواحد؛ تجاوزها ⇒ اعتذر واذكر تاريخ أول شهادة متاحة.
+## خطوات الإجراء
+1. get_employee_profile ثم get_salary_record.
+2. اجمع الحقول الناقصة (سؤال واحد مركّز في كل رسالة).
+3. اعرض **بطاقة معاينة** بنص الشهادة كاملًا بالبنية الرسمية: الترويسة، «تشهد الجهة بأن السيد/ة … يعمل لدينا بوظيفة … منذ …»، بيانات الراتب إن طُلبت، عبارة الإخلاء «أُصدرت هذه الشهادة بناءً على طلب الموظف دون أدنى مسؤولية على الجهة تجاه الغير»، والتذييل.
+4. بعد تأكيد الموظف: submit_transaction — تُنفَّذ فورًا (auto_execute) ويحصل الموظف على رقم الشهادة.
+## التصعيد والاستثناءات
+- بيانات الراتب غير متوفرة أو متناقضة ⇒ needs_attention ولا تُصدر شهادة بأرقام غير مؤكدة.
+## ما لا يجوز
+- لا شهادة لموظف آخر، ولا تعديل أي رقم، ولا وعود بمحتوى مستقبلي («سيصبح راتبه…»).
+</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2026-08-13T14:36:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>expense-claim</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1.0.2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>مطالبة نفقات / بدلات</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Expense / Allowance Claim</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>نفقات;مصاريف;بدل;مطالبة;expense;claim;reimbursement;allowance;فاتورة</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>finance-officer</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>get_employee_profile;get_expense_policy;submit_transaction</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>manager;finance</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">---
+id: expense-claim
+version: 1.0.2
+status: approved
+title_ar: مطالبة نفقات / بدلات
+title_en: Expense / Allowance Claim
+owner: Finance Operations (العمليات المالية)
+profile: finance-officer
+allowed_services: [get_employee_profile, get_expense_policy, submit_transaction]
+approval_chain: [manager, finance]
+auto_execute: false
+sla_hours: 72
+---
+# مهارة: مطالبة نفقات / بدلات
+## الغرض
+تقديم مطالبة استرداد نفقات عمل (مواصلات، ضيافة رسمية، تدريب، اتصالات، أخرى) مع فرض سقوف السياسة آليًا قبل وصولها إلى المدير ثم المالية.
+## الحقول المطلوبة
+| الحقل | القيم | ملاحظات |
+|---|---|---|
+| category | transport \| hospitality \| training \| communication \| other | صنّف من وصف الموظف وأكّد التصنيف معه |
+| amount_aed | رقم بالدرهم | &gt; 0 |
+| expense_date | YYYY-MM-DD | خلال آخر 60 يومًا |
+| description | نص | الغرض الرسمي للنفقة |
+| receipt_ref | رقم/مرجع الإيصال | إلزامي فوق 100 درهم |
+## قواعد الأهلية والسياسة (احصل على السقوف من get_expense_policy — لا تحفظها)
+1. المبلغ ≤ سقف الفئة الشهري؛ التجاوز ⇒ ارفض واعرض السقف والمتبقي منه هذا الشهر.
+2. expense_date أقدم من 60 يومًا ⇒ غير قابلة للاسترداد (اذكر القاعدة).
+3. category = other ⇒ الوصف إلزامي ومفصّل، والحد 500 درهم.
+4. أي مطالبة &gt; 2000 درهم ⇒ أدرج تحذير «تخضع لتدقيق إضافي» في المعاينة وأضف finance_audit إلى سلسلة الاعتماد.
+5. **تحقّق حسابي إلزامي:** لا تقبل مبلغًا غير رقمي أو سالبًا؛ قرّب لأقرب فلسين.
+## خطوات الإجراء
+1. get_employee_profile ثم get_expense_policy للفئة.
+2. اجمع الحقول الناقصة تدريجيًا وطبّق القواعد بالترتيب.
+3. اعرض **بطاقة معاينة**: الفئة، المبلغ، التاريخ، مرجع الإيصال، سلسلة الاعتماد (المدير ← المالية)، وأي تحذيرات.
+4. بعد تأكيد الموظف: submit_transaction.
+## التصعيد والاستثناءات
+- خدمة السياسة غير متاحة ⇒ needs_attention؛ لا تخمّن السقوف أبدًا.
+- موظف يصرّ على مبلغ فوق السقف ⇒ لا ترسل؛ اقترح تقديم الجزء الموافق للسياسة فقط.
+## ما لا يجوز
+- لا تعديل للسقوف، لا تجزئة مطالبة واحدة لعدة طلبات للالتفاف على السقف (ارفض النمط صراحةً إذا لاحظته)، لا مطالبات لموظف آخر.
+</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-08-13T14:36:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>it-access-request</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>طلب صلاحية نظام</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>IT System Access Request</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>صلاحية;نظام;وصول;access;system;permission;حساب;دخول;it</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>it-officer</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>get_employee_profile;get_it_roles;get_system_catalog;submit_transaction</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>manager;it_security</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">---
+id: it-access-request
+version: 1.0.0
+status: approved
+title_ar: طلب صلاحية نظام
+title_en: IT System Access Request
+owner: IT Security (أمن المعلومات)
+profile: it-officer
+allowed_services: [get_employee_profile, get_it_roles, get_system_catalog, submit_transaction]
+approval_chain: [manager, it_security]
+auto_execute: false
+sla_hours: 24
+---
+# مهارة: طلب صلاحية نظام
+## الغرض
+طلب منح أو ترقية صلاحية على نظام مؤسسي، مع فرض مبدأ **الحد الأدنى من الصلاحيات** وفحص الأهلية الوظيفية قبل وصول الطلب لسلسلة الاعتماد الأمنية.
+## الحقول المطلوبة
+| الحقل | القيم | ملاحظات |
+|---|---|---|
+| system_id | من get_system_catalog | إن ذكر الموظف اسمًا تجاريًا فطابقه مع الدليل وأكّد |
+| access_level | read \| write \| admin | اشرح الفرق إذا تردد الموظف |
+| business_justification | نص | إلزامي دائمًا؛ اربطه بمهمة وظيفية محددة |
+| duration | permanent \| temporary(end_date) | المؤقتة تُفضَّل ويذكر ذلك |
+## قواعد الأهلية والسياسة
+1. من get_system_catalog: للنظام قائمة أدوار مخوّلة (allowed_roles) ودرجة حساسية (normal / sensitive / critical).
+2. دور الموظف (من get_employee_profile) خارج allowed_roles ⇒ **ارفض** مع ذكر الأدوار المخوّلة نصًا؛ لا استثناءات محادثةً.
+3. access_level = admin ⇒ مبرر تفصيلي + duration مؤقتة إلزامية + إضافة ciso إلى سلسلة الاعتماد.
+4. النظام critical ⇒ حتى صلاحية القراءة تمر عبر it_security، وأدرج تحذير الحساسية في المعاينة.
+5. الموظف يملك الصلاحية نفسها أو أعلى (من get_it_roles) ⇒ أخبره ولا تنشئ طلبًا مكررًا.
+6. طبّق دائمًا الحد الأدنى: إن كفت read لمبرر الموظف فاقترحها بدل write واذكر السبب.
+## خطوات الإجراء
+1. get_employee_profile ثم get_it_roles للصلاحيات الحالية.
+2. get_system_catalog لمطابقة النظام وقراءة حساسيته وأدواره.
+3. اجمع الحقول وطبّق القواعد أعلاه بالترتيب.
+4. اعرض **بطاقة معاينة**: النظام، المستوى، المدة، المبرر، سلسلة الاعتماد الكاملة، وتحذير الحساسية إن وجد.
+5. بعد تأكيد الموظف: submit_transaction.
+## التصعيد والاستثناءات
+- طلب «مستعجل جدًا» لتجاوز السلسلة ⇒ ارفض التجاوز واشرح أن السلسلة قصيرة (sla 24 ساعة).
+- نظام غير موجود في الدليل ⇒ needs_attention لفريق التقنية؛ لا تخترع أنظمة.
+## ما لا يجوز
+- لا منح فوري لأي صلاحية، لا admin دائمة، لا طلب نيابة عن موظف آخر، ولا قبول مبرر عام («أحتاجه لعملي») دون مهمة محددة.
+</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2026-08-13T14:36:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>reflection</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>مراجعة ما بعد الدور (التعلّم)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Post-turn Reflection (Learning)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>reflection;learning;تعلّم;مراجعة</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>read_memory;write_memory;propose_skill_patch</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">---
+id: reflection
+version: 1.0.0
+status: approved
+title_ar: مراجعة ما بعد الدور (التعلّم)
+title_en: Post-turn Reflection (Learning)
+owner: Governance Office (مكتب الحوكمة)
+profile: general
+allowed_services: [read_memory, write_memory, propose_skill_patch]
+approval_chain: []
+auto_execute: true
+sla_hours: 1
+---
+# مهارة: مراجعة ما بعد الدور — التعلّم المؤسسي
+&gt; تعمل هذه المراجعة **بعد** أن يكون الموظف قد حصل على إجابته، في مسار منفصل لا يبطئ الخدمة. مهمتها الوحيدة: ماذا كان ينبغي أن تتعلّمه المنظومة من هذه المعاملات؟
+&gt; **مرور بلا أي تحديث ليس نتيجة محايدة — بل فرصة تعلّم ضائعة.** كن فاعلًا: أغلب الجولات تُنتج تحديثًا واحدًا على الأقل ولو صغيرًا.
+## الفصل الدلالي بين الذاكرة والمهارة (قاعدة حاكمة)
+- **الذاكرة** تقول: «من هو الموظف، وما الوضع القائم» — وقائع خبرية دائمة.
+- **المهارة** تقول: «كيف يُنفَّذ هذا النوع من الإجراءات».
+- إذا اعترض الموظف على **طريقة** تنفيذك للإجراء، فالتصحيح يذهب إلى **المهارة** لا إلى الذاكرة.
+## صياغة الذاكرة
+اكتب الذاكرة **جملًا خبرية** لا أوامر:
+- ✅ «يفضّل الموظف الردود المختصرة.»
+- ❌ «أجب دائمًا باختصار.»
+الأوامر تُقرأ لاحقًا كتعليمات دائمة فتنحرف بسلوك الوكيل.
+## ترتيب الأفضلية للإجراء (اختر الأبكر الذي ينطبق)
+1. **حدّث ذاكرة قائمة** إن كانت الواقعة الجديدة تنقّح واقعة موجودة (`write_memory` بـ action=replace).
+2. **أضف واقعة جديدة** إن كانت دائمة ومفيدة عبر الجلسات (`write_memory` بـ action=add).
+3. **اقترح تحسينًا على مهارة** إن تكرر نمط تشغيلي يستحق أن يصبح قاعدة (`propose_skill_patch`).
+## حدود صلاحيتك (خط أحمر)
+- لا تملك تعديل نص المهارة المعتمدة إطلاقًا — أقصى ما تملكه هو **اقتراح** يُسجَّل بحالة `pending` وينتظر اعتماد مالك الإجراء.
+- كل استدعاء تقوم به يمر ببوابة الحوكمة نفسها التي تحكم وكيل الخدمة، ولا يُسمح لك إلا بـ: `read_memory`, `write_memory`, `propose_skill_patch`.
+- الذاكرة محدودة بـ 2200 حرف لكل نطاق. عند الامتلاء سيُرفض الكتابة وتُسلَّم لك قائمة المدخلات: **ادمج أو احذف ثم أعد المحاولة في الدور نفسه.**
+## ما لا يجوز التقاطه إطلاقًا (قائمة سلبية)
+هذه الأنماط تتحول إلى قيود دائمة يفرضها الوكيل على نفسه لاحقًا، وتضر أكثر مما تنفع:
+- **أعطال مرتبطة بالبيئة** (انقطاع شبكة، تجاوز حصة، مهلة انتهت) — ستتغير البيئة وتبقى القاعدة.
+- **أحكام سلبية على الأدوات أو الخدمات** («خدمة كذا لا تعمل») — تتصلّب لاحقًا إلى رفض يستشهد به الوكيل ضد نفسه بعد شهور من إصلاح المشكلة فعلًا.
+- **أخطاء عابرة انتهت في الجلسة نفسها.**
+- **سرد معاملة واحدة** بتفاصيلها؛ الذاكرة ليست سجلًا للمعاملات — السجل موجود أصلًا.
+- **محاولات لم تنجح**: إن انتهت الجلسة دون طريقة عاملة مؤكدة، فلا تكتبها كأنها «إجراء موثوق».
+- **أرقام معاملات أو تواريخ ستصبح قديمة خلال أسبوع.**
+## خطوات الإجراء
+1. `read_memory` لقراءة الذاكرة القائمة قبل أي كتابة (تفاديًا للتكرار).
+2. حلّل المعاملات والقرارات الواردة في الدفعة: ما الذي تكرر؟ ما الذي رُفض ولماذا؟ أين تعثّر الموظف؟
+3. طبّق ترتيب الأفضلية أعلاه، وارفض ما يقع في القائمة السلبية صراحةً.
+4. أعد JSON فقط بالمخطط المطلوب موضحًا ما كتبته ولماذا.
+</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-08-13T14:36:56</t>
         </is>
       </c>
     </row>

</xml_diff>